<commit_message>
Task3: lion ages in list, age report and ageing
Lions get a random age from the list of possible ages; the list holds
the ages of all living lions and is updated by each lion every step
(remove previous age, age by one year, add current age). Dying lions
are removed. Number, min, mean and max of the ages are written to the
console and shown in monitors. Prompt log updated (rows 4-7).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Task3/PROMPT_LOG.xlsx
+++ b/Task3/PROMPT_LOG.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -579,6 +579,106 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>In the initialisation, add the age of all lions to the list; in a reflex, remove previous and add current age values</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Added lion attribute age &lt;- one_of(lion_ages); in init the list is emptied and filled with all lion ages (ask lion { add age to: lion_ages; })</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Agent first proposed a global reflex that rebuilds the whole list; corrected to each lion updating its own age. The planned lion reflex (remove previous, add current age) and the removal of dying lions were written but missing from the saved file; they were added again in step 6</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Each time step, report the number of values in the list, their minimum, mean and maximum</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Added global reflex report_lion_ages that writes n, min, mean and max of lion_ages to the console every cycle; added four monitors (number, minimum, mean, maximum lion age)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Reported in console and monitors (user's choice); empty-list check avoids errors when all lions are dead</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Lions also age each time step</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Added lion reflex update_age_in_list: removes the previous age from lion_ages, adds 1 year (age &lt;- age + 1), adds the current age; starve now removes the lion's age from the list before it dies</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>1 year per time step; no maximum age yet (lions older than 60 dying comes in a later step)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Commit and push, document in the log</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Committed and pushed steps 4–6 (lion ages in the list, age report, ageing) and both prompt logs to GitHub</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Agent checked before committing that all parts of steps 4–6 are in the saved file</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Task3: colour lions in shades of red by mean population age
Lion colour is a computed attribute blending light red (mean age 0) to
dark red (mean age 60+), so it always shows the current mean age, also
in the first picture. Prompt log updated (rows 8-10).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Task3/PROMPT_LOG.xlsx
+++ b/Task3/PROMPT_LOG.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -679,6 +679,81 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Colour the agents in shades of red according to the mean age of the population</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Lion color now updated every step with blend between dark red (139, 0, 0) and light red (255, 200, 200) from the mean of lion_ages (scale 0–60 years, capped); aspect comment changed from orange to red</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Only lions (only they have an age); all lions share the same shade. Without a maximum age the mean keeps rising, so lions soon become dark red</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>The first red shade should already be the current average</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Changed lion color from &lt;- #red update: blend(…) to the computed attribute color -&gt; blend(…), so it is recalculated whenever the lion is drawn</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Before, lions were plain red in the first picture until the first step; now the shade always matches the current mean age</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Commit and push, document in the log</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Committed and pushed steps 8–9 (lion colour by mean age) and both prompt logs to GitHub</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Task3: version numbering per commit (v3.3)
Each commit raises the model version by 0.1; earlier log rows set to
3.0-3.2 per commit, version added to the model header.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Task3/PROMPT_LOG.xlsx
+++ b/Task3/PROMPT_LOG.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -600,7 +600,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>3.1</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>3.1</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>3.1</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>3.1</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>3.2</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>3.2</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,32 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>3.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Increase the model version by 0.1 after each commit, also for earlier rows; version in the model header; matching Git tag per commit</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Set rows 4–7 to 3.1 and rows 8–10 to 3.2 (one version per commit); added * Version: 3.3 to the model header; tagged the earlier commits v3.0, v3.1, v3.2 and this commit v3.3</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>This commit counts as its own version (3.3); from now on every commit raises the version by 0.1</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>3.3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Task3: version per task step (v3.4)
Versions now follow the task steps: 3.0 age list, 3.1 lion ages and
update reflex incl. ageing, 3.2 age report, 3.3 red shades, 3.4 version
numbering. Log and model header updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Task3/PROMPT_LOG.xlsx
+++ b/Task3/PROMPT_LOG.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -625,7 +625,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>3.2</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>3.2</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>3.3</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>3.3</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>3.3</t>
         </is>
       </c>
     </row>
@@ -775,7 +775,32 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>3.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Version per task step instead of per commit: 3.0 age list, 3.1 ages in list + update reflex (incl. ageing), 3.2 age report, 3.3 red shades, 3.4 version numbering</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Re-set the version column accordingly; model header * Version: 3.4; moved tags v3.2 → bc28952 and v3.3 → f6ed04f, new tag v3.4</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Agent first counted one version per commit; corrected by the user. Commit and documentation rows keep the version of their step; row 7 is 3.2 because that commit completed steps 3.1 and 3.2</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>3.4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Task3: lions older than 60 die (v3.4)
New global max_lion_age (60) and lion reflex die_of_old_age, which
removes the lion's age from the list before it dies. The version
numbering is no longer counted as its own version. Prompt log updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Task3/PROMPT_LOG.xlsx
+++ b/Task3/PROMPT_LOG.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -775,7 +775,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>3.3</t>
         </is>
       </c>
     </row>
@@ -799,6 +799,56 @@
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Lions older than 60 die</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Added global variable max_lion_age &lt;- 60; new lion reflex die_of_old_age (after ageing, before starving) that removes the lion's age from the list and calls do die when age &gt; max_lion_age; header version 3.4</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Lions aged exactly 60 survive, at 61 they die. Without reproduction all lions are dead after at most 61 steps</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Commit and push, document; the version numbering is not an extra version</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Rows 11–12 (version numbering) set to 3.3, old-age death is now 3.4 (was 3.5); header * Version: 3.4; tag v3.4 moved from the numbering commit to this commit; committed and pushed</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Versions are only raised by model steps, not by documentation changes</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>

</xml_diff>

<commit_message>
Task3: baby lion born when an old lion dies (v3.5)
Just before a lion older than 60 dies, it creates a baby lion with age 0
at its location; the baby's age is added to the list. Prompt log updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Task3/PROMPT_LOG.xlsx
+++ b/Task3/PROMPT_LOG.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -854,6 +854,56 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Just before an old lion dies, a baby lion is born with age 0</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>In reflex die_of_old_age, before do die: create lion { age &lt;- 0; location &lt;- myself.location; add age to: lion_ages; }; header version 3.5</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Baby is born at the parent's location (user's choice) with the normal starting energy; only old-age deaths produce a baby, starving lions do not. Open: whether a newborn already ages in its birth step (min would then show 1)</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Commit and push, document in the log</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Committed and pushed the birth of baby lions and both prompt logs to GitHub; tagged v3.5</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Agent checked before committing that the birth code is in the saved file</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Task3: document GAMA test result in prompt log
All steps 3.0-3.5 run in GAMA; newborn lions start at age 0 and age
from the next step on.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Task3/PROMPT_LOG.xlsx
+++ b/Task3/PROMPT_LOG.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -904,6 +904,31 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Tested the model in GAMA</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>No code change; documented the test result and committed the log</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>All steps 3.0–3.5 run as expected in GAMA. Open point from row 15 resolved: a newborn lion is born with age 0 and only ages in the next step</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>